<commit_message>
Establish V2 audit pipeline and freeze current user inputs
</commit_message>
<xml_diff>
--- a/测产.xlsx
+++ b/测产.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\HNAAS\7-杨美眉paper\paper7 气候与成花诱导\数据分析\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cry\物候产量\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D58BEE5-5046-4716-B51D-0DC3D868CFBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AB3F210-C7E7-4DD5-B6D0-44D707F0FBB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13560" yWindow="2775" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="25">
   <si>
     <t>示范园</t>
   </si>
@@ -167,6 +167,10 @@
   </si>
   <si>
     <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t>A</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -441,14 +445,14 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -462,6 +466,66 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -479,66 +543,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -821,40 +825,40 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L47"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.5" customHeight="1" thickBot="1">
-      <c r="B1" s="40" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="40" t="s">
+    <row r="1" spans="1:12" ht="15.6" customHeight="1" thickBot="1">
+      <c r="B1" s="25" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40" t="s">
+      <c r="D1" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="42" t="s">
+      <c r="E1" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="43"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="40" t="s">
+      <c r="F1" s="37"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="40" t="s">
+      <c r="I1" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="40" t="s">
+      <c r="J1" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="40" t="s">
+      <c r="K1" s="25" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="14.5" thickBot="1">
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
+    <row r="2" spans="1:12" ht="15" thickBot="1">
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
       <c r="E2" s="1" t="s">
         <v>8</v>
       </c>
@@ -864,20 +868,20 @@
       <c r="G2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
-    </row>
-    <row r="3" spans="1:12" ht="14.5" thickBot="1">
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+    </row>
+    <row r="3" spans="1:12" ht="15" thickBot="1">
       <c r="A3" s="18">
         <v>2022</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="27" t="s">
         <v>11</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D3" s="3">
         <v>135</v>
@@ -900,13 +904,13 @@
       <c r="J3" s="3">
         <v>32.880000000000003</v>
       </c>
-      <c r="K3" s="31">
+      <c r="K3" s="30">
         <v>990</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="14.5" thickBot="1">
+    <row r="4" spans="1:12" ht="15" thickBot="1">
       <c r="A4" s="18"/>
-      <c r="B4" s="29"/>
+      <c r="B4" s="28"/>
       <c r="C4" s="2" t="s">
         <v>13</v>
       </c>
@@ -931,11 +935,11 @@
       <c r="J4" s="3">
         <v>27.12</v>
       </c>
-      <c r="K4" s="32"/>
-    </row>
-    <row r="5" spans="1:12" ht="14.5" thickBot="1">
+      <c r="K4" s="31"/>
+    </row>
+    <row r="5" spans="1:12" ht="15" thickBot="1">
       <c r="A5" s="18"/>
-      <c r="B5" s="30"/>
+      <c r="B5" s="29"/>
       <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
@@ -954,11 +958,11 @@
       <c r="J5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="33"/>
-    </row>
-    <row r="6" spans="1:12" ht="14.5" thickBot="1">
+      <c r="K5" s="32"/>
+    </row>
+    <row r="6" spans="1:12" ht="15" thickBot="1">
       <c r="A6" s="18"/>
-      <c r="B6" s="28" t="s">
+      <c r="B6" s="27" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -985,13 +989,13 @@
       <c r="J6" s="3">
         <v>131.59</v>
       </c>
-      <c r="K6" s="34">
+      <c r="K6" s="33">
         <v>1804.4</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="14.5" thickBot="1">
+    <row r="7" spans="1:12" ht="15" thickBot="1">
       <c r="A7" s="18"/>
-      <c r="B7" s="29"/>
+      <c r="B7" s="28"/>
       <c r="C7" s="2" t="s">
         <v>13</v>
       </c>
@@ -1016,11 +1020,11 @@
       <c r="J7" s="3">
         <v>126.18</v>
       </c>
-      <c r="K7" s="35"/>
-    </row>
-    <row r="8" spans="1:12" ht="14.5" thickBot="1">
+      <c r="K7" s="34"/>
+    </row>
+    <row r="8" spans="1:12" ht="15" thickBot="1">
       <c r="A8" s="18"/>
-      <c r="B8" s="30"/>
+      <c r="B8" s="29"/>
       <c r="C8" s="2" t="s">
         <v>14</v>
       </c>
@@ -1033,11 +1037,11 @@
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
-      <c r="K8" s="36"/>
-    </row>
-    <row r="9" spans="1:12" ht="14.5" thickBot="1">
+      <c r="K8" s="35"/>
+    </row>
+    <row r="9" spans="1:12" ht="15" thickBot="1">
       <c r="A9" s="18"/>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="27" t="s">
         <v>17</v>
       </c>
       <c r="C9" s="5" t="s">
@@ -1064,13 +1068,13 @@
       <c r="J9" s="6">
         <v>116.35</v>
       </c>
-      <c r="K9" s="37">
+      <c r="K9" s="39">
         <v>1691.64</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="14.5" thickBot="1">
+    <row r="10" spans="1:12" ht="15" thickBot="1">
       <c r="A10" s="18"/>
-      <c r="B10" s="29"/>
+      <c r="B10" s="28"/>
       <c r="C10" s="2" t="s">
         <v>13</v>
       </c>
@@ -1095,11 +1099,11 @@
       <c r="J10" s="3">
         <v>82.66</v>
       </c>
-      <c r="K10" s="38"/>
-    </row>
-    <row r="11" spans="1:12" ht="14.5" thickBot="1">
+      <c r="K10" s="40"/>
+    </row>
+    <row r="11" spans="1:12" ht="15" thickBot="1">
       <c r="A11" s="18"/>
-      <c r="B11" s="30"/>
+      <c r="B11" s="29"/>
       <c r="C11" s="2" t="s">
         <v>14</v>
       </c>
@@ -1112,13 +1116,13 @@
       </c>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
-      <c r="K11" s="39"/>
-    </row>
-    <row r="12" spans="1:12" ht="14.5" thickBot="1">
+      <c r="K11" s="41"/>
+    </row>
+    <row r="12" spans="1:12" ht="15" thickBot="1">
       <c r="A12" s="18">
         <v>2023</v>
       </c>
-      <c r="B12" s="28" t="s">
+      <c r="B12" s="27" t="s">
         <v>11</v>
       </c>
       <c r="C12" s="5" t="s">
@@ -1145,14 +1149,14 @@
       <c r="J12" s="6">
         <v>50.88</v>
       </c>
-      <c r="K12" s="31">
+      <c r="K12" s="30">
         <v>1590</v>
       </c>
       <c r="L12" s="7"/>
     </row>
-    <row r="13" spans="1:12" ht="14.5" thickBot="1">
+    <row r="13" spans="1:12" ht="15" thickBot="1">
       <c r="A13" s="18"/>
-      <c r="B13" s="29"/>
+      <c r="B13" s="28"/>
       <c r="C13" s="2" t="s">
         <v>13</v>
       </c>
@@ -1177,12 +1181,12 @@
       <c r="J13" s="3">
         <v>44.12</v>
       </c>
-      <c r="K13" s="32"/>
+      <c r="K13" s="31"/>
       <c r="L13" s="7"/>
     </row>
-    <row r="14" spans="1:12" ht="14.5" thickBot="1">
+    <row r="14" spans="1:12" ht="15" thickBot="1">
       <c r="A14" s="18"/>
-      <c r="B14" s="30"/>
+      <c r="B14" s="29"/>
       <c r="C14" s="2" t="s">
         <v>14</v>
       </c>
@@ -1201,12 +1205,12 @@
       <c r="J14" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="K14" s="33"/>
+      <c r="K14" s="32"/>
       <c r="L14" s="7"/>
     </row>
-    <row r="15" spans="1:12" ht="14.5" thickBot="1">
+    <row r="15" spans="1:12" ht="15" thickBot="1">
       <c r="A15" s="18"/>
-      <c r="B15" s="28" t="s">
+      <c r="B15" s="27" t="s">
         <v>16</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -1233,14 +1237,14 @@
       <c r="J15" s="3">
         <v>54.09</v>
       </c>
-      <c r="K15" s="34">
+      <c r="K15" s="33">
         <v>753.6</v>
       </c>
       <c r="L15" s="7"/>
     </row>
-    <row r="16" spans="1:12" ht="14.5" thickBot="1">
+    <row r="16" spans="1:12" ht="15" thickBot="1">
       <c r="A16" s="18"/>
-      <c r="B16" s="29"/>
+      <c r="B16" s="28"/>
       <c r="C16" s="2" t="s">
         <v>13</v>
       </c>
@@ -1265,12 +1269,12 @@
       <c r="J16" s="3">
         <v>52.18</v>
       </c>
-      <c r="K16" s="35"/>
+      <c r="K16" s="34"/>
       <c r="L16" s="7"/>
     </row>
-    <row r="17" spans="1:12" ht="14.5" thickBot="1">
+    <row r="17" spans="1:12" ht="15" thickBot="1">
       <c r="A17" s="18"/>
-      <c r="B17" s="30"/>
+      <c r="B17" s="29"/>
       <c r="C17" s="2" t="s">
         <v>14</v>
       </c>
@@ -1283,12 +1287,12 @@
       </c>
       <c r="I17" s="3"/>
       <c r="J17" s="3"/>
-      <c r="K17" s="36"/>
+      <c r="K17" s="35"/>
       <c r="L17" s="7"/>
     </row>
-    <row r="18" spans="1:12" ht="14.5" thickBot="1">
+    <row r="18" spans="1:12" ht="15" thickBot="1">
       <c r="A18" s="18"/>
-      <c r="B18" s="28" t="s">
+      <c r="B18" s="27" t="s">
         <v>17</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -1315,14 +1319,14 @@
       <c r="J18" s="3">
         <v>50.35</v>
       </c>
-      <c r="K18" s="37">
+      <c r="K18" s="39">
         <v>783.55</v>
       </c>
       <c r="L18" s="7"/>
     </row>
-    <row r="19" spans="1:12" ht="14.5" thickBot="1">
+    <row r="19" spans="1:12" ht="15" thickBot="1">
       <c r="A19" s="18"/>
-      <c r="B19" s="29"/>
+      <c r="B19" s="28"/>
       <c r="C19" s="2" t="s">
         <v>13</v>
       </c>
@@ -1347,12 +1351,12 @@
       <c r="J19" s="3">
         <v>45.66</v>
       </c>
-      <c r="K19" s="38"/>
+      <c r="K19" s="40"/>
       <c r="L19" s="7"/>
     </row>
-    <row r="20" spans="1:12" ht="14.5" thickBot="1">
+    <row r="20" spans="1:12" ht="15" thickBot="1">
       <c r="A20" s="18"/>
-      <c r="B20" s="30"/>
+      <c r="B20" s="29"/>
       <c r="C20" s="2" t="s">
         <v>14</v>
       </c>
@@ -1365,10 +1369,10 @@
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
-      <c r="K20" s="39"/>
+      <c r="K20" s="41"/>
       <c r="L20" s="7"/>
     </row>
-    <row r="21" spans="1:12" ht="14.5" thickBot="1">
+    <row r="21" spans="1:12" ht="15" thickBot="1">
       <c r="A21" s="18">
         <v>2024</v>
       </c>
@@ -1399,11 +1403,11 @@
       <c r="J21" s="9">
         <v>21.83</v>
       </c>
-      <c r="K21" s="25">
+      <c r="K21" s="45">
         <v>718.74</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="14.5" thickBot="1">
+    <row r="22" spans="1:12" ht="15" thickBot="1">
       <c r="A22" s="18"/>
       <c r="B22" s="20"/>
       <c r="C22" s="10" t="s">
@@ -1430,9 +1434,9 @@
       <c r="J22" s="11">
         <v>21.29</v>
       </c>
-      <c r="K22" s="26"/>
-    </row>
-    <row r="23" spans="1:12" ht="14.5" thickBot="1">
+      <c r="K22" s="46"/>
+    </row>
+    <row r="23" spans="1:12" ht="15" thickBot="1">
       <c r="A23" s="18"/>
       <c r="B23" s="21"/>
       <c r="C23" s="10" t="s">
@@ -1459,9 +1463,9 @@
       <c r="J23" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="K23" s="27"/>
-    </row>
-    <row r="24" spans="1:12" ht="14.5" thickBot="1">
+      <c r="K23" s="47"/>
+    </row>
+    <row r="24" spans="1:12" ht="15" thickBot="1">
       <c r="A24" s="18"/>
       <c r="B24" s="19" t="s">
         <v>16</v>
@@ -1490,11 +1494,11 @@
       <c r="J24" s="11">
         <v>8.16</v>
       </c>
-      <c r="K24" s="15">
+      <c r="K24" s="22">
         <v>107.14</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="14.5" thickBot="1">
+    <row r="25" spans="1:12" ht="15" thickBot="1">
       <c r="A25" s="18"/>
       <c r="B25" s="20"/>
       <c r="C25" s="10" t="s">
@@ -1521,9 +1525,9 @@
       <c r="J25" s="11">
         <v>7.63</v>
       </c>
-      <c r="K25" s="16"/>
-    </row>
-    <row r="26" spans="1:12" ht="14.5" thickBot="1">
+      <c r="K25" s="23"/>
+    </row>
+    <row r="26" spans="1:12" ht="15" thickBot="1">
       <c r="A26" s="18"/>
       <c r="B26" s="21"/>
       <c r="C26" s="10" t="s">
@@ -1548,9 +1552,9 @@
       <c r="J26" s="11">
         <v>7.35</v>
       </c>
-      <c r="K26" s="17"/>
-    </row>
-    <row r="27" spans="1:12" ht="14.5" thickBot="1">
+      <c r="K26" s="24"/>
+    </row>
+    <row r="27" spans="1:12" ht="15" thickBot="1">
       <c r="A27" s="18"/>
       <c r="B27" s="19" t="s">
         <v>17</v>
@@ -1579,11 +1583,11 @@
       <c r="J27" s="9">
         <v>61.76</v>
       </c>
-      <c r="K27" s="22">
+      <c r="K27" s="42">
         <v>1027.8</v>
       </c>
     </row>
-    <row r="28" spans="1:12" ht="14.5" thickBot="1">
+    <row r="28" spans="1:12" ht="15" thickBot="1">
       <c r="A28" s="18"/>
       <c r="B28" s="20"/>
       <c r="C28" s="10" t="s">
@@ -1610,9 +1614,9 @@
       <c r="J28" s="11">
         <v>61.58</v>
       </c>
-      <c r="K28" s="23"/>
-    </row>
-    <row r="29" spans="1:12" ht="14.5" thickBot="1">
+      <c r="K28" s="43"/>
+    </row>
+    <row r="29" spans="1:12" ht="15" thickBot="1">
       <c r="A29" s="18"/>
       <c r="B29" s="21"/>
       <c r="C29" s="10" t="s">
@@ -1639,9 +1643,9 @@
       <c r="J29" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="K29" s="24"/>
-    </row>
-    <row r="30" spans="1:12" ht="14.5" thickBot="1">
+      <c r="K29" s="44"/>
+    </row>
+    <row r="30" spans="1:12" ht="15" thickBot="1">
       <c r="A30" s="18">
         <v>2025</v>
       </c>
@@ -1672,11 +1676,11 @@
       <c r="J30" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="K30" s="15" t="s">
+      <c r="K30" s="22" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="14.5" thickBot="1">
+    <row r="31" spans="1:12" ht="15" thickBot="1">
       <c r="A31" s="18"/>
       <c r="B31" s="20"/>
       <c r="C31" s="10" t="s">
@@ -1703,9 +1707,9 @@
       <c r="J31" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="K31" s="16"/>
-    </row>
-    <row r="32" spans="1:12" ht="14.5" thickBot="1">
+      <c r="K31" s="23"/>
+    </row>
+    <row r="32" spans="1:12" ht="15" thickBot="1">
       <c r="A32" s="18"/>
       <c r="B32" s="21"/>
       <c r="C32" s="10" t="s">
@@ -1732,9 +1736,9 @@
       <c r="J32" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="K32" s="17"/>
-    </row>
-    <row r="33" spans="1:11" ht="14.5" thickBot="1">
+      <c r="K32" s="24"/>
+    </row>
+    <row r="33" spans="1:11" ht="15" thickBot="1">
       <c r="A33" s="18"/>
       <c r="B33" s="19" t="s">
         <v>16</v>
@@ -1763,11 +1767,11 @@
       <c r="J33" s="13">
         <v>33.549999999999997</v>
       </c>
-      <c r="K33" s="15">
+      <c r="K33" s="22">
         <v>450.14</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="14.5" thickBot="1">
+    <row r="34" spans="1:11" ht="15" thickBot="1">
       <c r="A34" s="18"/>
       <c r="B34" s="20"/>
       <c r="C34" s="10" t="s">
@@ -1794,9 +1798,9 @@
       <c r="J34" s="14">
         <v>31.12</v>
       </c>
-      <c r="K34" s="16"/>
-    </row>
-    <row r="35" spans="1:11" ht="14.5" thickBot="1">
+      <c r="K34" s="23"/>
+    </row>
+    <row r="35" spans="1:11" ht="15" thickBot="1">
       <c r="A35" s="18"/>
       <c r="B35" s="21"/>
       <c r="C35" s="10" t="s">
@@ -1821,9 +1825,9 @@
       <c r="J35" s="14">
         <v>31.78</v>
       </c>
-      <c r="K35" s="17"/>
-    </row>
-    <row r="36" spans="1:11" ht="14.5" thickBot="1">
+      <c r="K35" s="24"/>
+    </row>
+    <row r="36" spans="1:11" ht="15" thickBot="1">
       <c r="A36" s="18"/>
       <c r="B36" s="19" t="s">
         <v>17</v>
@@ -1852,11 +1856,11 @@
       <c r="J36" s="9">
         <v>71.760000000000005</v>
       </c>
-      <c r="K36" s="15">
+      <c r="K36" s="22">
         <v>1205.8800000000001</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="14.5" thickBot="1">
+    <row r="37" spans="1:11" ht="15" thickBot="1">
       <c r="A37" s="18"/>
       <c r="B37" s="20"/>
       <c r="C37" s="10" t="s">
@@ -1883,9 +1887,9 @@
       <c r="J37" s="11">
         <v>70.099999999999994</v>
       </c>
-      <c r="K37" s="16"/>
-    </row>
-    <row r="38" spans="1:11" ht="14.5" thickBot="1">
+      <c r="K37" s="23"/>
+    </row>
+    <row r="38" spans="1:11" ht="15" thickBot="1">
       <c r="A38" s="18"/>
       <c r="B38" s="21"/>
       <c r="C38" s="10" t="s">
@@ -1912,11 +1916,11 @@
       <c r="J38" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="K38" s="17"/>
-    </row>
-    <row r="39" spans="1:11" ht="14.5" thickBot="1">
+      <c r="K38" s="24"/>
+    </row>
+    <row r="39" spans="1:11" ht="15" thickBot="1">
       <c r="A39" s="18">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B39" s="19" t="s">
         <v>11</v>
@@ -1930,26 +1934,26 @@
       <c r="E39" s="9">
         <v>38.450000000000003</v>
       </c>
-      <c r="F39" s="45">
+      <c r="F39" s="15">
         <v>44.21</v>
       </c>
       <c r="G39" s="9">
         <v>37.369999999999997</v>
       </c>
-      <c r="H39" s="45">
+      <c r="H39" s="15">
         <v>22.18</v>
       </c>
       <c r="I39" s="9">
         <v>0</v>
       </c>
-      <c r="J39" s="45">
+      <c r="J39" s="15">
         <v>40.01</v>
       </c>
-      <c r="K39" s="15">
+      <c r="K39" s="22">
         <v>1306.23</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="14.5" thickBot="1">
+    <row r="40" spans="1:11" ht="15" thickBot="1">
       <c r="A40" s="18"/>
       <c r="B40" s="20"/>
       <c r="C40" s="10" t="s">
@@ -1976,9 +1980,9 @@
       <c r="J40" s="12">
         <v>31.82</v>
       </c>
-      <c r="K40" s="16"/>
-    </row>
-    <row r="41" spans="1:11" ht="14.5" thickBot="1">
+      <c r="K40" s="23"/>
+    </row>
+    <row r="41" spans="1:11" ht="15" thickBot="1">
       <c r="A41" s="18"/>
       <c r="B41" s="21"/>
       <c r="C41" s="10" t="s">
@@ -1995,9 +1999,9 @@
       </c>
       <c r="I41" s="11"/>
       <c r="J41" s="11"/>
-      <c r="K41" s="17"/>
-    </row>
-    <row r="42" spans="1:11" ht="14.5" thickBot="1">
+      <c r="K41" s="24"/>
+    </row>
+    <row r="42" spans="1:11" ht="15" thickBot="1">
       <c r="A42" s="18"/>
       <c r="B42" s="19" t="s">
         <v>16</v>
@@ -2011,26 +2015,26 @@
       <c r="E42" s="13">
         <v>60.11</v>
       </c>
-      <c r="F42" s="45">
+      <c r="F42" s="15">
         <v>55.68</v>
       </c>
-      <c r="G42" s="45">
+      <c r="G42" s="15">
         <v>60.04</v>
       </c>
-      <c r="H42" s="45">
+      <c r="H42" s="15">
         <v>18.350000000000001</v>
       </c>
       <c r="I42" s="9">
         <v>0</v>
       </c>
-      <c r="J42" s="45">
+      <c r="J42" s="15">
         <v>58.61</v>
       </c>
-      <c r="K42" s="15">
+      <c r="K42" s="22">
         <v>750.25</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="14.5" thickBot="1">
+    <row r="43" spans="1:11" ht="15" thickBot="1">
       <c r="A43" s="18"/>
       <c r="B43" s="20"/>
       <c r="C43" s="10" t="s">
@@ -2057,9 +2061,9 @@
       <c r="J43" s="12">
         <v>52.7</v>
       </c>
-      <c r="K43" s="16"/>
-    </row>
-    <row r="44" spans="1:11" ht="14.5" thickBot="1">
+      <c r="K43" s="23"/>
+    </row>
+    <row r="44" spans="1:11" ht="15" thickBot="1">
       <c r="A44" s="18"/>
       <c r="B44" s="21"/>
       <c r="C44" s="10" t="s">
@@ -2074,9 +2078,9 @@
       <c r="H44" s="12"/>
       <c r="I44" s="11"/>
       <c r="J44" s="12"/>
-      <c r="K44" s="17"/>
-    </row>
-    <row r="45" spans="1:11" ht="14.5" thickBot="1">
+      <c r="K44" s="24"/>
+    </row>
+    <row r="45" spans="1:11" ht="15" thickBot="1">
       <c r="A45" s="18"/>
       <c r="B45" s="19" t="s">
         <v>17</v>
@@ -2087,13 +2091,13 @@
       <c r="D45" s="9">
         <v>170</v>
       </c>
-      <c r="E45" s="46">
+      <c r="E45" s="16">
         <v>71.67</v>
       </c>
-      <c r="F45" s="45">
+      <c r="F45" s="15">
         <v>76.23</v>
       </c>
-      <c r="G45" s="45">
+      <c r="G45" s="15">
         <v>77.88</v>
       </c>
       <c r="H45" s="9">
@@ -2105,11 +2109,11 @@
       <c r="J45" s="9">
         <v>75.260000000000005</v>
       </c>
-      <c r="K45" s="15">
+      <c r="K45" s="22">
         <v>1205.8800000000001</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="14.5" thickBot="1">
+    <row r="46" spans="1:11" ht="15" thickBot="1">
       <c r="A46" s="18"/>
       <c r="B46" s="20"/>
       <c r="C46" s="10" t="s">
@@ -2118,7 +2122,7 @@
       <c r="D46" s="11">
         <v>30</v>
       </c>
-      <c r="E46" s="47">
+      <c r="E46" s="17">
         <v>50.78</v>
       </c>
       <c r="F46" s="12">
@@ -2136,9 +2140,9 @@
       <c r="J46" s="11">
         <v>55.88</v>
       </c>
-      <c r="K46" s="16"/>
-    </row>
-    <row r="47" spans="1:11" ht="14.5" thickBot="1">
+      <c r="K46" s="23"/>
+    </row>
+    <row r="47" spans="1:11" ht="15" thickBot="1">
       <c r="A47" s="18"/>
       <c r="B47" s="21"/>
       <c r="C47" s="10" t="s">
@@ -2159,39 +2163,10 @@
       <c r="J47" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="K47" s="17"/>
+      <c r="K47" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="A39:A47"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="K39:K41"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="K42:K44"/>
-    <mergeCell ref="B45:B47"/>
-    <mergeCell ref="K45:K47"/>
-    <mergeCell ref="J1:J2"/>
-    <mergeCell ref="K1:K2"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="K3:K5"/>
-    <mergeCell ref="B6:B8"/>
-    <mergeCell ref="K6:K8"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:G1"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="K9:K11"/>
-    <mergeCell ref="B12:B14"/>
-    <mergeCell ref="B15:B17"/>
-    <mergeCell ref="A3:A11"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="K12:K14"/>
-    <mergeCell ref="K15:K17"/>
-    <mergeCell ref="K18:K20"/>
-    <mergeCell ref="A12:A20"/>
     <mergeCell ref="B27:B29"/>
     <mergeCell ref="K27:K29"/>
     <mergeCell ref="A21:A29"/>
@@ -2206,6 +2181,35 @@
     <mergeCell ref="K33:K35"/>
     <mergeCell ref="B36:B38"/>
     <mergeCell ref="K36:K38"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="K12:K14"/>
+    <mergeCell ref="K15:K17"/>
+    <mergeCell ref="K18:K20"/>
+    <mergeCell ref="A12:A20"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="K9:K11"/>
+    <mergeCell ref="B12:B14"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="A3:A11"/>
+    <mergeCell ref="J1:J2"/>
+    <mergeCell ref="K1:K2"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="K3:K5"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="K6:K8"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:G1"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="A39:A47"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="K39:K41"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="K42:K44"/>
+    <mergeCell ref="B45:B47"/>
+    <mergeCell ref="K45:K47"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>